<commit_message>
balance: the tutorials name the Bathroom Slippers for Double EXP
Two boxes of the lessons (Lesson.pck BattleTeacher_11-12, Teaching.pck
CheatsTeaching_19) named the Slave's Torc, whose row W042 was dropped;
the Bathroom Slippers (P090) give Double EXP. The sheet About says the
build writes them.
</commit_message>
<xml_diff>
--- a/data_tables/balance_tutorial_text.xlsx
+++ b/data_tables/balance_tutorial_text.xlsx
@@ -438,7 +438,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>The tutorial texts of the Balance variant: lines of the lessons of Euthys (Lesson.pck) and of the library (Teaching.pck). They state figures of the Balance variant, so they belong to that build and never to the QoL one. Nothing builds them yet: tools/build_variant.py has no Balance variant.</t>
+          <t>The tutorial texts of the Balance variant: lines of the lessons of Euthys (Lesson.pck) and of the library (Teaching.pck). They state figures of the Balance variant, so they belong to that build and never to the QoL one. tools/build_variant.py balance writes them into Lesson.pck and Teaching.pck.</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>"Simply equip her with the Slave's Torc to double her gains.
+          <t>"Simply equip her with the Bathroom Slippers to double her gains.
 She will soak up so much experience from stronger monsters that
 she'll rejoin the vanguard before you even have time to complain."</t>
         </is>
@@ -873,7 +873,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>True on the Balance variant only (row W042)</t>
+          <t>True on the Balance variant only (row P090)</t>
         </is>
       </c>
     </row>
@@ -1663,8 +1663,8 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Equip training accessories like Slave's Torc to double
-experience gains, rapidly catching up allies who underwent resets.
+          <t>Equip the Bathroom Slippers to double experience gains,
+rapidly catching up allies who underwent resets.
 Facing higher-level monsters also grants native bonus EXP.</t>
         </is>
       </c>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>True on the Balance variant only: row W042 gives the Slave's Torc Double EXP; the gap factors are 0x450739</t>
+          <t>True on the Balance variant only: row P090 gives the Bathroom Slippers Double EXP; the gap factors are 0x450739</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(tutorials): limit line 3 width to avoid next-page prompt overlap
</commit_message>
<xml_diff>
--- a/data_tables/balance_tutorial_text.xlsx
+++ b/data_tables/balance_tutorial_text.xlsx
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -548,6 +548,21 @@
       <c r="C3" t="inlineStr">
         <is>
           <t>Characters of a line: the originals reach 75 in Lesson.pck and 69 in Teaching.pck</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>max_width_line3</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>65</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Characters of line 3: 5 less than max_width to prevent overlap with the next-page prompt button</t>
         </is>
       </c>
     </row>
@@ -624,7 +639,7 @@
         <is>
           <t>"Pay close attention: heavy 2H blades and rifles hit hard,
 but their severe delay leaves you wide open!
-Have them Defend to advance their gauge and recover the initiative."</t>
+Have them Defend to raise their gauge and regain initiative."</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -664,7 +679,7 @@
         <is>
           <t>"Mid-range spears and whips ignore penalties from adjacent rows,
 while bows and magic strike across all rows at full power.
-Position your allies wisely, Fried, lest you suffer needless harm."</t>
+Position allies wisely, Fried, lest you suffer needless harm."</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -705,7 +720,7 @@
         <is>
           <t>"Precisely! Stacking 100 resistance also cuts elemental damage in half.
 Combine this with a Paladin's Cover or a Dark Lord's leeching,
-and your front line will stand firm even against divine magic."</t>
+and your front line will stand firm against divine magic."</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -858,7 +873,7 @@
         <is>
           <t>"Simply equip her with the Bathroom Slippers to double her gains.
 She will soak up so much experience from stronger monsters that
-she'll rejoin the vanguard before you even have time to complain."</t>
+she'll rejoin the vanguard before you can even complain."</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -898,7 +913,7 @@
         <is>
           <t>"I visit often. A hearty meal restores you before a journey,
 and the finest dishes send you off with Brave, Protect or
-the three physical guards already cast. Exquisite and practical."</t>
+three physical guards already cast. Exquisite and practical."</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1878,7 +1893,7 @@
         <is>
           <t>When level resetting, if the gap is 59 or greater between
 your former level and the level you reset to, all stats and
-resistances increase by +1 permanently, building toward Crown EX.</t>
+resistances gain +1 permanently, building toward Crown EX.</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">

</xml_diff>

<commit_message>
feat(teaching): add comprehensive in-game guides for all classes
</commit_message>
<xml_diff>
--- a/data_tables/balance_tutorial_text.xlsx
+++ b/data_tables/balance_tutorial_text.xlsx
@@ -1454,12 +1454,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>checked</t>
+          <t>held</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0x44cd3b, 0x44eff9: x1.5 from blows and spells; 0x47ea6b: any damage wakes; 0x44af7e: hit for certain</t>
+          <t>Superseded by full merged tutorial in tools/class_tutorial_text.py</t>
         </is>
       </c>
     </row>
@@ -1489,12 +1489,12 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>checked</t>
+          <t>held</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Was "200 res = 100% immune": the enchantment sum stops at 100 (0x4f8490), so 200 is not a figure a player can plan on. Half a percent per point and the block at 100 are read (0x652b64, 0x481fc2)</t>
+          <t>Superseded by full Intermediate Classes guide in tools/class_tutorial_text.py</t>
         </is>
       </c>
     </row>
@@ -1826,12 +1826,12 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>checked</t>
+          <t>held</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>EnemyAIData: scripts switch sets on the HP share of the enemy (FORMULAS 9, source 0)</t>
+          <t>Superseded by full merged tutorial in tools/class_tutorial_text.py</t>
         </is>
       </c>
     </row>
@@ -1862,12 +1862,12 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>checked</t>
+          <t>held</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Barrage Rondo, Provoke with Dark Aura and the critical second roll all exist as named</t>
+          <t>Superseded by full Advanced Classes guide in tools/class_tutorial_text.py</t>
         </is>
       </c>
     </row>

</xml_diff>